<commit_message>
Corrige rastreabilidade da validacao do TP03
</commit_message>
<xml_diff>
--- a/atividades/TP03-sinais/planilha-tp03.xlsx
+++ b/atividades/TP03-sinais/planilha-tp03.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\etc\Projetos do Marcelinho\SistemasAutomatizados\tmp\tp03-planilha-qa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F632D1D6-B3C2-42EF-8171-08500212F4AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74EF7C2F-1474-4FD6-9CC7-858E732A415A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumo" sheetId="1" r:id="rId1"/>
@@ -200,9 +200,6 @@
     <t>Limitações da simulação</t>
   </si>
   <si>
-    <t>• Wokwi e planilha validam lógica, escalonamento, quantização, transições e documentação.</t>
-  </si>
-  <si>
     <t>• Não validam tolerância real do resistor, ruído eletromagnético, aterramento, isolamento ou corrente física de um laço 4–20 mA.</t>
   </si>
   <si>
@@ -452,12 +449,6 @@
     <t>tempC = pct nesta faixa</t>
   </si>
   <si>
-    <t>Dados brutos — aquisição simulada</t>
-  </si>
-  <si>
-    <t>Somente entradas observadas. Cálculos e classificações ficam na aba Analise.</t>
-  </si>
-  <si>
     <t>Amostra</t>
   </si>
   <si>
@@ -473,9 +464,6 @@
     <t>Observação</t>
   </si>
   <si>
-    <t>Wokwi (simulação)</t>
-  </si>
-  <si>
     <t>mínimo</t>
   </si>
   <si>
@@ -786,6 +774,18 @@
   </si>
   <si>
     <t>G7</t>
+  </si>
+  <si>
+    <t>código escolhido</t>
+  </si>
+  <si>
+    <t>Dados brutos — amostras de teste</t>
+  </si>
+  <si>
+    <t>• A planilha e a verificação nativa validam cálculos, escalonamento, quantização, transições e documentação; o circuito público no Wokwi foi conferido estruturalmente.</t>
+  </si>
+  <si>
+    <t>Códigos escolhidos para cobrir a faixa e as transições; não são capturas do Monitor Serial.</t>
   </si>
 </sst>
 </file>
@@ -966,7 +966,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1005,18 +1005,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1429,6 +1432,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="pt-BR"/>
               <a:t>Tendência da temperatura simulada</a:t>
             </a:r>
           </a:p>
@@ -2044,6 +2048,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="pt-BR"/>
                   <a:t>Amostra</a:t>
                 </a:r>
               </a:p>
@@ -2082,6 +2087,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="pt-BR"/>
                   <a:t>Temperatura simulada (°C)</a:t>
                 </a:r>
               </a:p>
@@ -2779,7 +2785,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -2791,8 +2797,8 @@
       <c r="I1" s="8"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
-        <v>230</v>
+      <c r="A2" s="21" t="s">
+        <v>226</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2805,36 +2811,36 @@
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B5" s="3">
         <v>3.2</v>
@@ -2855,7 +2861,7 @@
         <v>FALHA ELETRICA</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="H5" s="3">
         <f>Parametros!$B$10+C5/100*(Parametros!$B$11-Parametros!$B$10)</f>
@@ -2868,7 +2874,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B6" s="3">
         <v>4</v>
@@ -2889,7 +2895,7 @@
         <v>FAIXA VALIDA</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="H6" s="3">
         <f>Parametros!$B$10+C6/100*(Parametros!$B$11-Parametros!$B$10)</f>
@@ -2902,7 +2908,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B7" s="3">
         <v>12</v>
@@ -2923,7 +2929,7 @@
         <v>FAIXA VALIDA</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="H7" s="3">
         <f>Parametros!$B$10+C7/100*(Parametros!$B$11-Parametros!$B$10)</f>
@@ -2936,7 +2942,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B8" s="3">
         <v>15.2</v>
@@ -2957,7 +2963,7 @@
         <v>FAIXA VALIDA</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="H8" s="3">
         <f>Parametros!$B$10+C8/100*(Parametros!$B$11-Parametros!$B$10)</f>
@@ -2970,7 +2976,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="B9" s="3">
         <v>17.600000000000001</v>
@@ -2991,7 +2997,7 @@
         <v>FAIXA VALIDA</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="H9" s="3">
         <f>Parametros!$B$10+C9/100*(Parametros!$B$11-Parametros!$B$10)</f>
@@ -3004,7 +3010,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B10" s="3">
         <v>20</v>
@@ -3025,7 +3031,7 @@
         <v>FAIXA VALIDA</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="H10" s="3">
         <f>Parametros!$B$10+C10/100*(Parametros!$B$11-Parametros!$B$10)</f>
@@ -3038,7 +3044,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B11" s="3">
         <v>20.8</v>
@@ -3059,7 +3065,7 @@
         <v>FALHA ELETRICA</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="H11" s="3">
         <f>Parametros!$B$10+C11/100*(Parametros!$B$11-Parametros!$B$10)</f>
@@ -3146,7 +3152,7 @@
       <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="17" t="s">
         <v>25</v>
       </c>
       <c r="B4" s="8"/>
@@ -3158,7 +3164,7 @@
       <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="17" t="s">
         <v>26</v>
       </c>
       <c r="B5" s="8"/>
@@ -3170,7 +3176,7 @@
       <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="17" t="s">
         <v>27</v>
       </c>
       <c r="B6" s="8"/>
@@ -3182,7 +3188,7 @@
       <c r="H6" s="8"/>
     </row>
     <row r="7" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="17" t="s">
         <v>28</v>
       </c>
       <c r="B7" s="8"/>
@@ -3194,7 +3200,7 @@
       <c r="H7" s="8"/>
     </row>
     <row r="8" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="17" t="s">
         <v>29</v>
       </c>
       <c r="B8" s="8"/>
@@ -3206,7 +3212,7 @@
       <c r="H8" s="8"/>
     </row>
     <row r="9" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="17" t="s">
         <v>30</v>
       </c>
       <c r="B9" s="8"/>
@@ -3233,15 +3239,15 @@
       <c r="A12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -3354,8 +3360,8 @@
       <c r="H21" s="8"/>
     </row>
     <row r="22" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
-        <v>48</v>
+      <c r="A22" s="17" t="s">
+        <v>242</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -3366,8 +3372,8 @@
       <c r="H22" s="8"/>
     </row>
     <row r="23" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
-        <v>49</v>
+      <c r="A23" s="17" t="s">
+        <v>48</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -3378,8 +3384,8 @@
       <c r="H23" s="8"/>
     </row>
     <row r="24" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
-        <v>50</v>
+      <c r="A24" s="17" t="s">
+        <v>49</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -3390,8 +3396,8 @@
       <c r="H24" s="8"/>
     </row>
     <row r="25" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
-        <v>51</v>
+      <c r="A25" s="17" t="s">
+        <v>50</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -3402,8 +3408,8 @@
       <c r="H25" s="8"/>
     </row>
     <row r="26" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
-        <v>52</v>
+      <c r="A26" s="17" t="s">
+        <v>51</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -3415,7 +3421,7 @@
     </row>
     <row r="27" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -3426,8 +3432,8 @@
       <c r="H27" s="8"/>
     </row>
     <row r="28" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="18" t="s">
-        <v>54</v>
+      <c r="A28" s="15" t="s">
+        <v>53</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -3439,31 +3445,31 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="B15:H15"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="B19:H19"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A3:H3"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="A9:H9"/>
     <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.45" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
@@ -3489,7 +3495,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -3497,170 +3503,170 @@
     </row>
     <row r="3" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" s="1">
         <v>0</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B5" s="1">
         <v>1023</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B6" s="1">
         <v>0</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B7" s="1">
         <v>100</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B8" s="1">
         <v>4</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B9" s="1">
         <v>20</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B10" s="1">
         <v>0</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B11" s="1">
         <v>10</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B12" s="1">
         <v>70</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B13" s="1">
         <v>85</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -3698,7 +3704,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -3709,163 +3715,163 @@
     </row>
     <row r="3" spans="1:7" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -3901,37 +3907,37 @@
   <sheetData>
     <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>132</v>
+        <v>241</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
       <c r="E1" s="8"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
+        <v>243</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
     </row>
     <row r="4" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -3945,10 +3951,10 @@
         <v>0</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -3962,10 +3968,10 @@
         <v>256</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -3979,10 +3985,10 @@
         <v>512</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -3996,10 +4002,10 @@
         <v>650</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -4013,10 +4019,10 @@
         <v>716</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -4030,10 +4036,10 @@
         <v>717</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -4047,10 +4053,10 @@
         <v>768</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4064,10 +4070,10 @@
         <v>830</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -4081,10 +4087,10 @@
         <v>869</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -4098,10 +4104,10 @@
         <v>870</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -4115,10 +4121,10 @@
         <v>950</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -4132,10 +4138,10 @@
         <v>1023</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -4149,10 +4155,10 @@
         <v>900</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -4166,10 +4172,10 @@
         <v>800</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -4183,10 +4189,10 @@
         <v>700</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>139</v>
+        <v>240</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -4240,7 +4246,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -4258,7 +4264,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -4276,25 +4282,25 @@
     </row>
     <row r="4" spans="1:14" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>42</v>
@@ -4303,19 +4309,19 @@
         <v>9</v>
       </c>
       <c r="J4" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N4" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -5255,7 +5261,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -5272,7 +5278,7 @@
     </row>
     <row r="3" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -5281,24 +5287,24 @@
     </row>
     <row r="4" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B5" s="3">
         <v>-1</v>
@@ -5317,7 +5323,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B6" s="3">
         <v>0</v>
@@ -5336,7 +5342,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B7" s="3">
         <v>69.989999999999995</v>
@@ -5355,7 +5361,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B8" s="3">
         <v>70</v>
@@ -5374,7 +5380,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B9" s="3">
         <v>84.99</v>
@@ -5393,7 +5399,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B10" s="3">
         <v>85</v>
@@ -5412,7 +5418,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B11" s="3">
         <v>100</v>
@@ -5431,7 +5437,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B12" s="3">
         <v>100.01</v>
@@ -5450,7 +5456,7 @@
     </row>
     <row r="16" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -5467,48 +5473,48 @@
     </row>
     <row r="17" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="M17" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B18" s="1">
         <v>0</v>
@@ -5548,7 +5554,7 @@
         <v>OFF</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="M18" s="1" t="str">
         <f t="shared" ref="M18:M26" si="3">IF(AND(E18&lt;0.0001,I18=J18,K18=L18),"CONFORME","REVISAR")</f>
@@ -5557,7 +5563,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B19" s="1">
         <v>256</v>
@@ -5597,7 +5603,7 @@
         <v>OFF</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="M19" s="1" t="str">
         <f t="shared" si="3"/>
@@ -5606,7 +5612,7 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B20" s="1">
         <v>512</v>
@@ -5646,7 +5652,7 @@
         <v>OFF</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="M20" s="1" t="str">
         <f t="shared" si="3"/>
@@ -5655,7 +5661,7 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B21" s="1">
         <v>716</v>
@@ -5695,7 +5701,7 @@
         <v>OFF</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="M21" s="1" t="str">
         <f t="shared" si="3"/>
@@ -5704,7 +5710,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B22" s="1">
         <v>717</v>
@@ -5744,7 +5750,7 @@
         <v>OFF</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="M22" s="1" t="str">
         <f t="shared" si="3"/>
@@ -5753,7 +5759,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B23" s="1">
         <v>768</v>
@@ -5793,7 +5799,7 @@
         <v>OFF</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="M23" s="1" t="str">
         <f t="shared" si="3"/>
@@ -5802,7 +5808,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B24" s="1">
         <v>869</v>
@@ -5842,7 +5848,7 @@
         <v>OFF</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="M24" s="1" t="str">
         <f t="shared" si="3"/>
@@ -5851,7 +5857,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B25" s="1">
         <v>870</v>
@@ -5891,7 +5897,7 @@
         <v>ON</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="M25" s="1" t="str">
         <f t="shared" si="3"/>
@@ -5900,7 +5906,7 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B26" s="1">
         <v>1023</v>
@@ -5940,7 +5946,7 @@
         <v>ON</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="M26" s="1" t="str">
         <f t="shared" si="3"/>
@@ -6026,7 +6032,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -6037,8 +6043,8 @@
       <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
-        <v>201</v>
+      <c r="A2" s="21" t="s">
+        <v>197</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -6050,33 +6056,33 @@
     </row>
     <row r="4" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>171</v>
-      </c>
       <c r="G4" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B5" s="1">
         <v>500</v>
@@ -6107,7 +6113,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B6" s="1">
         <v>504</v>
@@ -6138,7 +6144,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B7" s="1">
         <v>498</v>
@@ -6169,7 +6175,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="B8" s="1">
         <v>502</v>
@@ -6200,7 +6206,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B9" s="1">
         <v>500</v>
@@ -6231,7 +6237,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B10" s="1">
         <v>620</v>
@@ -6262,7 +6268,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B11" s="1">
         <v>504</v>
@@ -6293,7 +6299,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B12" s="1">
         <v>498</v>
@@ -6324,7 +6330,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="B13" s="1">
         <v>502</v>
@@ -6355,7 +6361,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B14" s="1">
         <v>500</v>
@@ -6386,7 +6392,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="B15" s="1">
         <v>500</v>
@@ -6461,7 +6467,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -6473,8 +6479,8 @@
       <c r="I1" s="8"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
-        <v>218</v>
+      <c r="A2" s="21" t="s">
+        <v>214</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -6487,36 +6493,36 @@
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B5" s="3">
         <v>0</v>
@@ -6552,7 +6558,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B6" s="3">
         <v>25</v>
@@ -6588,7 +6594,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B7" s="3">
         <v>50</v>
@@ -6624,7 +6630,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B8" s="3">
         <v>75</v>
@@ -6660,7 +6666,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B9" s="3">
         <v>100</v>

</xml_diff>